<commit_message>
#16 Supplier link added in eSpark BOM
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/eSpark_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/eSpark_BOM_v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="215">
   <si>
     <t>Component list</t>
   </si>
@@ -661,6 +661,9 @@
   </si>
   <si>
     <t xml:space="preserve">Glass Pipe </t>
+  </si>
+  <si>
+    <t>Digikey</t>
   </si>
 </sst>
 </file>
@@ -1984,7 +1987,9 @@
       <c r="J10" s="37" t="s">
         <v>173</v>
       </c>
-      <c r="K10" s="37"/>
+      <c r="K10" s="37" t="s">
+        <v>173</v>
+      </c>
       <c r="L10" s="37">
         <v>1</v>
       </c>
@@ -1995,11 +2000,15 @@
       <c r="N10" s="37">
         <v>6</v>
       </c>
-      <c r="O10" s="61"/>
-      <c r="P10" s="38"/>
+      <c r="O10" s="61" t="s">
+        <v>214</v>
+      </c>
+      <c r="P10" s="38">
+        <v>1.59</v>
+      </c>
       <c r="Q10" s="38">
         <f>P10*N10</f>
-        <v>0</v>
+        <v>9.5400000000000009</v>
       </c>
       <c r="R10" s="63" t="s">
         <v>182</v>
@@ -2046,12 +2055,18 @@
         <f t="shared" ref="M11" si="1">L11*5</f>
         <v>5</v>
       </c>
-      <c r="N11" s="51"/>
-      <c r="O11" s="60"/>
-      <c r="P11" s="52"/>
+      <c r="N11" s="51">
+        <v>100</v>
+      </c>
+      <c r="O11" s="60" t="s">
+        <v>174</v>
+      </c>
+      <c r="P11" s="52">
+        <v>4.0000000000000001E-3</v>
+      </c>
       <c r="Q11" s="52">
         <f t="shared" ref="Q11" si="2">P11*N11</f>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R11" s="51"/>
       <c r="S11" s="51"/>
@@ -3727,7 +3742,7 @@
       <c r="P42" s="74"/>
       <c r="Q42" s="48">
         <f>SUM(Q10:Q41)</f>
-        <v>198.68480000000002</v>
+        <v>208.62480000000002</v>
       </c>
       <c r="R42" s="69"/>
       <c r="S42" s="70"/>
@@ -3753,7 +3768,7 @@
       <c r="P43" s="74"/>
       <c r="Q43" s="49">
         <f>Q42/5</f>
-        <v>39.736960000000003</v>
+        <v>41.724960000000003</v>
       </c>
       <c r="R43" s="71"/>
       <c r="S43" s="72"/>
@@ -3794,9 +3809,11 @@
     <hyperlink ref="O36" r:id="rId25"/>
     <hyperlink ref="O23" r:id="rId26"/>
     <hyperlink ref="O14" r:id="rId27"/>
+    <hyperlink ref="O10" r:id="rId28"/>
+    <hyperlink ref="O11" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId28"/>
-  <drawing r:id="rId29"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>
+  <drawing r:id="rId31"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#16 eSpark BOM updated.
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/eSpark_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/eSpark_BOM_v2.0.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2130" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2135" uniqueCount="241">
   <si>
     <t>Component list</t>
   </si>
@@ -578,9 +578,6 @@
     <t>LTE_MODULE_v2.0</t>
   </si>
   <si>
-    <t>JLCPCB</t>
-  </si>
-  <si>
     <t>HJ Tech</t>
   </si>
   <si>
@@ -747,6 +744,9 @@
   </si>
   <si>
     <t>Total Cost (1000 Boards)</t>
+  </si>
+  <si>
+    <t>Chipsmall</t>
   </si>
 </sst>
 </file>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -2346,22 +2346,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="E10" s="37" t="s">
         <v>194</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>195</v>
       </c>
       <c r="F10" s="37" t="s">
         <v>171</v>
       </c>
       <c r="G10" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H10" s="37" t="s">
         <v>196</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>197</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>172</v>
@@ -2383,7 +2383,7 @@
         <v>6</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P10" s="38">
         <v>1.59</v>
@@ -2410,13 +2410,13 @@
         <v>19</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>71</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H11" s="51" t="s">
         <v>113</v>
@@ -2425,10 +2425,10 @@
         <v>172</v>
       </c>
       <c r="J11" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="K11" s="51" t="s">
         <v>200</v>
-      </c>
-      <c r="K11" s="51" t="s">
-        <v>201</v>
       </c>
       <c r="L11" s="51">
         <v>1</v>
@@ -2519,7 +2519,7 @@
         <v>9</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E13" s="51" t="s">
         <v>45</v>
@@ -2578,22 +2578,22 @@
         <v>21</v>
       </c>
       <c r="E14" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="F14" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="G14" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="G14" s="37" t="s">
+      <c r="H14" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="H14" s="37" t="s">
+      <c r="I14" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="J14" s="37" t="s">
         <v>189</v>
-      </c>
-      <c r="I14" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="J14" s="37" t="s">
-        <v>190</v>
       </c>
       <c r="K14" s="37" t="s">
         <v>151</v>
@@ -3076,28 +3076,28 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="H23" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="I23" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J23" s="51" t="s">
         <v>219</v>
-      </c>
-      <c r="H23" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="I23" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J23" s="51" t="s">
-        <v>220</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -3245,7 +3245,7 @@
         <v>13</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E26" s="37" t="s">
         <v>56</v>
@@ -3410,7 +3410,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="53" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>35</v>
@@ -3469,7 +3469,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -3581,7 +3581,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -3795,7 +3795,7 @@
       <c r="R35" s="51"/>
       <c r="S35" s="59"/>
     </row>
-    <row r="36" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="47">
         <f t="shared" si="0"/>
@@ -3823,7 +3823,7 @@
         <v>172</v>
       </c>
       <c r="J36" s="51" t="s">
-        <v>145</v>
+        <v>172</v>
       </c>
       <c r="K36" s="51" t="s">
         <v>172</v>
@@ -3839,14 +3839,14 @@
         <v>6</v>
       </c>
       <c r="O36" s="61" t="s">
-        <v>184</v>
+        <v>240</v>
       </c>
       <c r="P36" s="52">
-        <v>27.036000000000001</v>
+        <v>62.987000000000002</v>
       </c>
       <c r="Q36" s="52">
         <f t="shared" ref="Q36" si="25">P36*N36</f>
-        <v>162.21600000000001</v>
+        <v>377.92200000000003</v>
       </c>
       <c r="R36" s="51"/>
       <c r="S36" s="59"/>
@@ -3917,7 +3917,7 @@
         <v>17</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>68</v>
@@ -4032,22 +4032,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>210</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>211</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>212</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -4088,20 +4088,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="68" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F41" s="68"/>
       <c r="G41" s="68" t="s">
+        <v>212</v>
+      </c>
+      <c r="H41" s="68" t="s">
         <v>213</v>
       </c>
-      <c r="H41" s="68" t="s">
-        <v>214</v>
-      </c>
       <c r="I41" s="68" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="68" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K41" s="68" t="s">
         <v>172</v>
@@ -4142,7 +4142,7 @@
       <c r="E42" s="51"/>
       <c r="F42" s="51"/>
       <c r="G42" s="51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H42" s="51"/>
       <c r="I42" s="51"/>
@@ -4178,7 +4178,7 @@
       <c r="P43" s="85"/>
       <c r="Q43" s="48">
         <f>SUM(Q10:Q42)</f>
-        <v>217.11340000000001</v>
+        <v>432.81939999999997</v>
       </c>
       <c r="R43" s="80"/>
       <c r="S43" s="81"/>
@@ -4204,7 +4204,7 @@
       <c r="P44" s="85"/>
       <c r="Q44" s="49">
         <f>Q43/5</f>
-        <v>43.42268</v>
+        <v>86.563879999999997</v>
       </c>
       <c r="R44" s="82"/>
       <c r="S44" s="83"/>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -4500,19 +4500,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>221</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>222</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>223</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>224</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -4528,22 +4528,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="E10" s="37" t="s">
         <v>194</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>195</v>
       </c>
       <c r="F10" s="37" t="s">
         <v>171</v>
       </c>
       <c r="G10" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H10" s="37" t="s">
         <v>196</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>197</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>172</v>
@@ -4565,7 +4565,7 @@
         <v>21</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P10" s="38">
         <v>1.431</v>
@@ -4592,13 +4592,13 @@
         <v>19</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>71</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H11" s="51" t="s">
         <v>113</v>
@@ -4607,10 +4607,10 @@
         <v>172</v>
       </c>
       <c r="J11" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="K11" s="51" t="s">
         <v>200</v>
-      </c>
-      <c r="K11" s="51" t="s">
-        <v>201</v>
       </c>
       <c r="L11" s="51">
         <v>1</v>
@@ -4701,7 +4701,7 @@
         <v>9</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E13" s="51" t="s">
         <v>45</v>
@@ -4760,22 +4760,22 @@
         <v>21</v>
       </c>
       <c r="E14" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="F14" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="G14" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="G14" s="37" t="s">
+      <c r="H14" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="H14" s="37" t="s">
+      <c r="I14" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="J14" s="37" t="s">
         <v>189</v>
-      </c>
-      <c r="I14" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="J14" s="37" t="s">
-        <v>190</v>
       </c>
       <c r="K14" s="37" t="s">
         <v>151</v>
@@ -5258,28 +5258,28 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="H23" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="I23" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J23" s="51" t="s">
         <v>219</v>
-      </c>
-      <c r="H23" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="I23" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J23" s="51" t="s">
-        <v>220</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -5427,7 +5427,7 @@
         <v>13</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E26" s="37" t="s">
         <v>56</v>
@@ -5592,7 +5592,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="53" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>35</v>
@@ -5651,7 +5651,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -5763,7 +5763,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -5977,7 +5977,7 @@
       <c r="R35" s="51"/>
       <c r="S35" s="59"/>
     </row>
-    <row r="36" spans="1:19" s="75" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" s="75" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="73"/>
       <c r="B36" s="47">
         <f t="shared" si="0"/>
@@ -6020,11 +6020,15 @@
       <c r="N36" s="51">
         <v>21</v>
       </c>
-      <c r="O36" s="61"/>
-      <c r="P36" s="52"/>
+      <c r="O36" s="61" t="s">
+        <v>240</v>
+      </c>
+      <c r="P36" s="52">
+        <v>47.240250000000003</v>
+      </c>
       <c r="Q36" s="52">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>992.04525000000012</v>
       </c>
       <c r="R36" s="51"/>
       <c r="S36" s="59"/>
@@ -6095,7 +6099,7 @@
         <v>17</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>68</v>
@@ -6210,22 +6214,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>210</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>211</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>212</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -6266,20 +6270,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>212</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>214</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -6320,7 +6324,7 @@
       <c r="E42" s="51"/>
       <c r="F42" s="51"/>
       <c r="G42" s="51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H42" s="51"/>
       <c r="I42" s="51"/>
@@ -6356,7 +6360,7 @@
       <c r="P43" s="85"/>
       <c r="Q43" s="48">
         <f>SUM(Q10:Q42)</f>
-        <v>151.11170000000001</v>
+        <v>1143.1569500000003</v>
       </c>
       <c r="R43" s="80"/>
       <c r="S43" s="81"/>
@@ -6382,7 +6386,7 @@
       <c r="P44" s="85"/>
       <c r="Q44" s="49">
         <f>Q43/20</f>
-        <v>7.5555850000000007</v>
+        <v>57.157847500000017</v>
       </c>
       <c r="R44" s="82"/>
       <c r="S44" s="83"/>
@@ -6425,9 +6429,10 @@
     <hyperlink ref="O40" r:id="rId27"/>
     <hyperlink ref="O41" r:id="rId28"/>
     <hyperlink ref="O23" r:id="rId29"/>
+    <hyperlink ref="O36" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId30"/>
+  <drawing r:id="rId31"/>
 </worksheet>
 </file>
 
@@ -6486,7 +6491,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -6676,19 +6681,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>224</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>225</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>226</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>227</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>228</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -6704,22 +6709,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="E10" s="37" t="s">
         <v>194</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>195</v>
       </c>
       <c r="F10" s="37" t="s">
         <v>171</v>
       </c>
       <c r="G10" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H10" s="37" t="s">
         <v>196</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>197</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>172</v>
@@ -6741,7 +6746,7 @@
         <v>51</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P10" s="38">
         <v>1.35</v>
@@ -6768,13 +6773,13 @@
         <v>19</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>71</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H11" s="51" t="s">
         <v>113</v>
@@ -6783,10 +6788,10 @@
         <v>172</v>
       </c>
       <c r="J11" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="K11" s="51" t="s">
         <v>200</v>
-      </c>
-      <c r="K11" s="51" t="s">
-        <v>201</v>
       </c>
       <c r="L11" s="51">
         <v>1</v>
@@ -6877,7 +6882,7 @@
         <v>9</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E13" s="51" t="s">
         <v>45</v>
@@ -6936,22 +6941,22 @@
         <v>21</v>
       </c>
       <c r="E14" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="F14" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="G14" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="G14" s="37" t="s">
+      <c r="H14" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="H14" s="37" t="s">
+      <c r="I14" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="J14" s="37" t="s">
         <v>189</v>
-      </c>
-      <c r="I14" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="J14" s="37" t="s">
-        <v>190</v>
       </c>
       <c r="K14" s="37" t="s">
         <v>151</v>
@@ -7434,28 +7439,28 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="H23" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="I23" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J23" s="51" t="s">
         <v>219</v>
-      </c>
-      <c r="H23" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="I23" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J23" s="51" t="s">
-        <v>220</v>
       </c>
       <c r="K23" s="51"/>
       <c r="L23" s="51">
@@ -7601,7 +7606,7 @@
         <v>13</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E26" s="37" t="s">
         <v>56</v>
@@ -7766,7 +7771,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="53" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>35</v>
@@ -7825,7 +7830,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -7937,7 +7942,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -8151,7 +8156,7 @@
       <c r="R35" s="51"/>
       <c r="S35" s="59"/>
     </row>
-    <row r="36" spans="1:19" s="75" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" s="75" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="73"/>
       <c r="B36" s="47">
         <f t="shared" si="0"/>
@@ -8194,11 +8199,15 @@
       <c r="N36" s="51">
         <v>51</v>
       </c>
-      <c r="O36" s="61"/>
-      <c r="P36" s="52"/>
+      <c r="O36" s="61" t="s">
+        <v>240</v>
+      </c>
+      <c r="P36" s="52">
+        <v>40.941549999999999</v>
+      </c>
       <c r="Q36" s="52">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2088.0190499999999</v>
       </c>
       <c r="R36" s="51"/>
       <c r="S36" s="59"/>
@@ -8269,7 +8278,7 @@
         <v>17</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>68</v>
@@ -8384,22 +8393,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>210</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>211</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>212</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -8440,20 +8449,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>212</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>214</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -8494,7 +8503,7 @@
       <c r="E42" s="51"/>
       <c r="F42" s="51"/>
       <c r="G42" s="51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H42" s="51"/>
       <c r="I42" s="51"/>
@@ -8530,7 +8539,7 @@
       <c r="P43" s="85"/>
       <c r="Q43" s="48">
         <f>SUM(Q10:Q42)</f>
-        <v>328.23919999999998</v>
+        <v>2416.2582500000003</v>
       </c>
       <c r="R43" s="80"/>
       <c r="S43" s="81"/>
@@ -8556,7 +8565,7 @@
       <c r="P44" s="85"/>
       <c r="Q44" s="49">
         <f>Q43/50</f>
-        <v>6.5647839999999995</v>
+        <v>48.325165000000005</v>
       </c>
       <c r="R44" s="82"/>
       <c r="S44" s="83"/>
@@ -8599,9 +8608,10 @@
     <hyperlink ref="O40" r:id="rId27"/>
     <hyperlink ref="O41" r:id="rId28"/>
     <hyperlink ref="O23" r:id="rId29"/>
+    <hyperlink ref="O36" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId30"/>
+  <drawing r:id="rId31"/>
 </worksheet>
 </file>
 
@@ -8660,7 +8670,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -8850,19 +8860,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>228</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>229</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>230</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>231</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>232</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -8878,22 +8888,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="E10" s="37" t="s">
         <v>194</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>195</v>
       </c>
       <c r="F10" s="37" t="s">
         <v>171</v>
       </c>
       <c r="G10" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H10" s="37" t="s">
         <v>196</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>197</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>172</v>
@@ -8915,7 +8925,7 @@
         <v>101</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P10" s="38">
         <v>1.1501999999999999</v>
@@ -8942,13 +8952,13 @@
         <v>19</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>71</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H11" s="51" t="s">
         <v>113</v>
@@ -8957,10 +8967,10 @@
         <v>172</v>
       </c>
       <c r="J11" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="K11" s="51" t="s">
         <v>200</v>
-      </c>
-      <c r="K11" s="51" t="s">
-        <v>201</v>
       </c>
       <c r="L11" s="51">
         <v>1</v>
@@ -9051,7 +9061,7 @@
         <v>9</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E13" s="51" t="s">
         <v>45</v>
@@ -9110,22 +9120,22 @@
         <v>21</v>
       </c>
       <c r="E14" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="F14" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="G14" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="G14" s="37" t="s">
+      <c r="H14" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="H14" s="37" t="s">
+      <c r="I14" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="J14" s="37" t="s">
         <v>189</v>
-      </c>
-      <c r="I14" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="J14" s="37" t="s">
-        <v>190</v>
       </c>
       <c r="K14" s="37" t="s">
         <v>151</v>
@@ -9608,28 +9618,28 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="H23" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="I23" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J23" s="51" t="s">
         <v>219</v>
-      </c>
-      <c r="H23" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="I23" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J23" s="51" t="s">
-        <v>220</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -9777,7 +9787,7 @@
         <v>13</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E26" s="37" t="s">
         <v>56</v>
@@ -9942,7 +9952,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="53" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>35</v>
@@ -10001,7 +10011,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -10113,7 +10123,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -10327,7 +10337,7 @@
       <c r="R35" s="51"/>
       <c r="S35" s="59"/>
     </row>
-    <row r="36" spans="1:19" s="75" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" s="75" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="73"/>
       <c r="B36" s="47">
         <f t="shared" si="0"/>
@@ -10367,12 +10377,18 @@
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="N36" s="51"/>
-      <c r="O36" s="61"/>
-      <c r="P36" s="52"/>
+      <c r="N36" s="51">
+        <v>101</v>
+      </c>
+      <c r="O36" s="61" t="s">
+        <v>240</v>
+      </c>
+      <c r="P36" s="52">
+        <v>36.21752</v>
+      </c>
       <c r="Q36" s="52">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>3657.9695200000001</v>
       </c>
       <c r="R36" s="51"/>
       <c r="S36" s="59"/>
@@ -10443,7 +10459,7 @@
         <v>17</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>68</v>
@@ -10558,22 +10574,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>210</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>211</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>212</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -10614,20 +10630,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>212</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>214</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -10668,7 +10684,7 @@
       <c r="E42" s="51"/>
       <c r="F42" s="51"/>
       <c r="G42" s="51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H42" s="51"/>
       <c r="I42" s="51"/>
@@ -10704,7 +10720,7 @@
       <c r="P43" s="85"/>
       <c r="Q43" s="48">
         <f>SUM(Q10:Q42)</f>
-        <v>594.2509</v>
+        <v>4252.2204199999996</v>
       </c>
       <c r="R43" s="80"/>
       <c r="S43" s="81"/>
@@ -10730,7 +10746,7 @@
       <c r="P44" s="85"/>
       <c r="Q44" s="49">
         <f>Q43/100</f>
-        <v>5.9425090000000003</v>
+        <v>42.522204199999997</v>
       </c>
       <c r="R44" s="82"/>
       <c r="S44" s="83"/>
@@ -10773,9 +10789,10 @@
     <hyperlink ref="O40" r:id="rId27"/>
     <hyperlink ref="O41" r:id="rId28"/>
     <hyperlink ref="O23" r:id="rId29"/>
+    <hyperlink ref="O36" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId30"/>
+  <drawing r:id="rId31"/>
 </worksheet>
 </file>
 
@@ -10834,7 +10851,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -11024,19 +11041,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>232</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>233</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>234</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>235</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>236</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -11052,22 +11069,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="E10" s="37" t="s">
         <v>194</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>195</v>
       </c>
       <c r="F10" s="37" t="s">
         <v>171</v>
       </c>
       <c r="G10" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H10" s="37" t="s">
         <v>196</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>197</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>172</v>
@@ -11089,7 +11106,7 @@
         <v>501</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P10" s="38">
         <v>0.94499999999999995</v>
@@ -11116,13 +11133,13 @@
         <v>19</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>71</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H11" s="51" t="s">
         <v>113</v>
@@ -11131,10 +11148,10 @@
         <v>172</v>
       </c>
       <c r="J11" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="K11" s="51" t="s">
         <v>200</v>
-      </c>
-      <c r="K11" s="51" t="s">
-        <v>201</v>
       </c>
       <c r="L11" s="51">
         <v>1</v>
@@ -11225,7 +11242,7 @@
         <v>9</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E13" s="51" t="s">
         <v>45</v>
@@ -11284,22 +11301,22 @@
         <v>21</v>
       </c>
       <c r="E14" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="F14" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="G14" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="G14" s="37" t="s">
+      <c r="H14" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="H14" s="37" t="s">
+      <c r="I14" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="J14" s="37" t="s">
         <v>189</v>
-      </c>
-      <c r="I14" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="J14" s="37" t="s">
-        <v>190</v>
       </c>
       <c r="K14" s="37" t="s">
         <v>151</v>
@@ -11782,28 +11799,28 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="H23" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="I23" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J23" s="51" t="s">
         <v>219</v>
-      </c>
-      <c r="H23" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="I23" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J23" s="51" t="s">
-        <v>220</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -11951,7 +11968,7 @@
         <v>13</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E26" s="37" t="s">
         <v>56</v>
@@ -12116,7 +12133,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="53" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>35</v>
@@ -12175,7 +12192,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -12287,7 +12304,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -12501,7 +12518,7 @@
       <c r="R35" s="51"/>
       <c r="S35" s="59"/>
     </row>
-    <row r="36" spans="1:19" s="75" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" s="75" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="73"/>
       <c r="B36" s="47">
         <f t="shared" si="0"/>
@@ -12541,14 +12558,18 @@
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="N36" s="51"/>
-      <c r="O36" s="61"/>
+      <c r="N36" s="51">
+        <v>501</v>
+      </c>
+      <c r="O36" s="61" t="s">
+        <v>240</v>
+      </c>
       <c r="P36" s="52">
-        <v>27.036000000000001</v>
+        <v>34.012979999999999</v>
       </c>
       <c r="Q36" s="52">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>17040.502980000001</v>
       </c>
       <c r="R36" s="51"/>
       <c r="S36" s="59"/>
@@ -12619,7 +12640,7 @@
         <v>17</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>68</v>
@@ -12734,22 +12755,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>210</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>211</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>212</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -12790,20 +12811,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>212</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>214</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -12844,7 +12865,7 @@
       <c r="E42" s="51"/>
       <c r="F42" s="51"/>
       <c r="G42" s="51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H42" s="51"/>
       <c r="I42" s="51"/>
@@ -12880,7 +12901,7 @@
       <c r="P43" s="85"/>
       <c r="Q43" s="48">
         <f>SUM(Q10:Q42)</f>
-        <v>2686.9485999999997</v>
+        <v>19727.451580000001</v>
       </c>
       <c r="R43" s="80"/>
       <c r="S43" s="81"/>
@@ -12906,7 +12927,7 @@
       <c r="P44" s="85"/>
       <c r="Q44" s="49">
         <f>Q43/500</f>
-        <v>5.3738971999999992</v>
+        <v>39.454903160000001</v>
       </c>
       <c r="R44" s="82"/>
       <c r="S44" s="83"/>
@@ -12949,9 +12970,10 @@
     <hyperlink ref="O40" r:id="rId27"/>
     <hyperlink ref="O41" r:id="rId28"/>
     <hyperlink ref="O23" r:id="rId29"/>
+    <hyperlink ref="O36" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId30"/>
+  <drawing r:id="rId31"/>
 </worksheet>
 </file>
 
@@ -13010,7 +13032,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -13200,19 +13222,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>236</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>237</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>238</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>239</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>240</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -13228,22 +13250,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="E10" s="37" t="s">
         <v>194</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>195</v>
       </c>
       <c r="F10" s="37" t="s">
         <v>171</v>
       </c>
       <c r="G10" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H10" s="37" t="s">
         <v>196</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>197</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>172</v>
@@ -13265,7 +13287,7 @@
         <v>1002</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P10" s="38">
         <v>0.78300000000000003</v>
@@ -13292,13 +13314,13 @@
         <v>19</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>71</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H11" s="51" t="s">
         <v>113</v>
@@ -13307,10 +13329,10 @@
         <v>172</v>
       </c>
       <c r="J11" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="K11" s="51" t="s">
         <v>200</v>
-      </c>
-      <c r="K11" s="51" t="s">
-        <v>201</v>
       </c>
       <c r="L11" s="51">
         <v>1</v>
@@ -13401,7 +13423,7 @@
         <v>9</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E13" s="51" t="s">
         <v>45</v>
@@ -13460,22 +13482,22 @@
         <v>21</v>
       </c>
       <c r="E14" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="F14" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="G14" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="G14" s="37" t="s">
+      <c r="H14" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="H14" s="37" t="s">
+      <c r="I14" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="J14" s="37" t="s">
         <v>189</v>
-      </c>
-      <c r="I14" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="J14" s="37" t="s">
-        <v>190</v>
       </c>
       <c r="K14" s="37" t="s">
         <v>151</v>
@@ -13958,28 +13980,28 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="H23" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="I23" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J23" s="51" t="s">
         <v>219</v>
-      </c>
-      <c r="H23" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="I23" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J23" s="51" t="s">
-        <v>220</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -14127,7 +14149,7 @@
         <v>13</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E26" s="37" t="s">
         <v>56</v>
@@ -14292,7 +14314,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="53" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>35</v>
@@ -14351,7 +14373,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -14463,7 +14485,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -14677,7 +14699,7 @@
       <c r="R35" s="51"/>
       <c r="S35" s="59"/>
     </row>
-    <row r="36" spans="1:19" s="75" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" s="75" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="73"/>
       <c r="B36" s="47">
         <f t="shared" si="0"/>
@@ -14717,12 +14739,18 @@
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N36" s="51"/>
-      <c r="O36" s="61"/>
-      <c r="P36" s="52"/>
+      <c r="N36" s="51">
+        <v>1001</v>
+      </c>
+      <c r="O36" s="61" t="s">
+        <v>240</v>
+      </c>
+      <c r="P36" s="52">
+        <v>31.493500000000001</v>
+      </c>
       <c r="Q36" s="52">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>31524.9935</v>
       </c>
       <c r="R36" s="51"/>
       <c r="S36" s="59"/>
@@ -14793,7 +14821,7 @@
         <v>17</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>68</v>
@@ -14908,22 +14936,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>210</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>211</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>212</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -14964,20 +14992,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>212</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>214</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -15018,7 +15046,7 @@
       <c r="E42" s="51"/>
       <c r="F42" s="51"/>
       <c r="G42" s="51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H42" s="51"/>
       <c r="I42" s="51"/>
@@ -15054,7 +15082,7 @@
       <c r="P43" s="85"/>
       <c r="Q43" s="48">
         <f>SUM(Q10:Q42)</f>
-        <v>5051.2368999999999</v>
+        <v>36576.230399999993</v>
       </c>
       <c r="R43" s="80"/>
       <c r="S43" s="81"/>
@@ -15080,7 +15108,7 @@
       <c r="P44" s="85"/>
       <c r="Q44" s="49">
         <f>Q43/1000</f>
-        <v>5.0512369000000001</v>
+        <v>36.576230399999993</v>
       </c>
       <c r="R44" s="82"/>
       <c r="S44" s="83"/>
@@ -15123,8 +15151,9 @@
     <hyperlink ref="O40" r:id="rId27"/>
     <hyperlink ref="O41" r:id="rId28"/>
     <hyperlink ref="O23" r:id="rId29"/>
+    <hyperlink ref="O36" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId30"/>
+  <drawing r:id="rId31"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#16 Extra Row Delete in BOM
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/eSpark_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/eSpark_BOM_v2.0.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2135" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2123" uniqueCount="240">
   <si>
     <t>Component list</t>
   </si>
@@ -636,9 +636,6 @@
   </si>
   <si>
     <t>Transistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glass Pipe </t>
   </si>
   <si>
     <t>Digikey</t>
@@ -2075,7 +2072,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -2383,7 +2380,7 @@
         <v>6</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P10" s="38">
         <v>1.59</v>
@@ -2400,7 +2397,7 @@
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="47">
-        <f t="shared" ref="B11:B42" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="54" t="s">
@@ -3076,19 +3073,19 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H23" s="51" t="s">
         <v>184</v>
@@ -3097,7 +3094,7 @@
         <v>172</v>
       </c>
       <c r="J23" s="51" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -3469,7 +3466,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -3581,7 +3578,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -3839,7 +3836,7 @@
         <v>6</v>
       </c>
       <c r="O36" s="61" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P36" s="52">
         <v>62.987000000000002</v>
@@ -4032,22 +4029,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>210</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>211</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -4088,20 +4085,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="68" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F41" s="68"/>
       <c r="G41" s="68" t="s">
+        <v>211</v>
+      </c>
+      <c r="H41" s="68" t="s">
         <v>212</v>
       </c>
-      <c r="H41" s="68" t="s">
-        <v>213</v>
-      </c>
       <c r="I41" s="68" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="68" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K41" s="68" t="s">
         <v>172</v>
@@ -4129,93 +4126,65 @@
       <c r="R41" s="68"/>
       <c r="S41" s="71"/>
     </row>
-    <row r="42" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="47">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>182</v>
-      </c>
-      <c r="D42" s="51"/>
-      <c r="E42" s="51"/>
-      <c r="F42" s="51"/>
-      <c r="G42" s="51" t="s">
-        <v>204</v>
-      </c>
-      <c r="H42" s="51"/>
-      <c r="I42" s="51"/>
-      <c r="J42" s="51"/>
-      <c r="K42" s="51"/>
-      <c r="L42" s="51"/>
-      <c r="M42" s="51"/>
-      <c r="N42" s="51"/>
-      <c r="O42" s="61"/>
-      <c r="P42" s="52"/>
-      <c r="Q42" s="52"/>
-      <c r="R42" s="51"/>
-      <c r="S42" s="39"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="O42" s="85"/>
+      <c r="P42" s="85"/>
+      <c r="Q42" s="48">
+        <f>SUM(Q10:Q41)</f>
+        <v>432.81939999999997</v>
+      </c>
+      <c r="R42" s="80"/>
+      <c r="S42" s="81"/>
     </row>
     <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="40"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="42"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="44"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="45"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="45"/>
-      <c r="L43" s="45"/>
-      <c r="M43" s="45"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
       <c r="N43" s="84" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O43" s="85"/>
       <c r="P43" s="85"/>
-      <c r="Q43" s="48">
-        <f>SUM(Q10:Q42)</f>
-        <v>432.81939999999997</v>
-      </c>
-      <c r="R43" s="80"/>
-      <c r="S43" s="81"/>
-    </row>
-    <row r="44" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="84" t="s">
-        <v>6</v>
-      </c>
-      <c r="O44" s="85"/>
-      <c r="P44" s="85"/>
-      <c r="Q44" s="49">
-        <f>Q43/5</f>
+      <c r="Q43" s="49">
+        <f>Q42/5</f>
         <v>86.563879999999997</v>
       </c>
-      <c r="R44" s="82"/>
-      <c r="S44" s="83"/>
+      <c r="R43" s="82"/>
+      <c r="S43" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="R43:S44"/>
+    <mergeCell ref="R42:S43"/>
+    <mergeCell ref="N42:P42"/>
     <mergeCell ref="N43:P43"/>
-    <mergeCell ref="N44:P44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O15" r:id="rId1"/>
@@ -4257,7 +4226,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -4500,19 +4469,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>219</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>220</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>221</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>221</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>222</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>223</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -4565,7 +4534,7 @@
         <v>21</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P10" s="38">
         <v>1.431</v>
@@ -4582,7 +4551,7 @@
     <row r="11" spans="1:19" s="75" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="73"/>
       <c r="B11" s="47">
-        <f t="shared" ref="B11:B42" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="54" t="s">
@@ -5258,19 +5227,19 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H23" s="51" t="s">
         <v>184</v>
@@ -5279,7 +5248,7 @@
         <v>172</v>
       </c>
       <c r="J23" s="51" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -5651,7 +5620,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -5763,7 +5732,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -6021,7 +5990,7 @@
         <v>21</v>
       </c>
       <c r="O36" s="61" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P36" s="52">
         <v>47.240250000000003</v>
@@ -6214,22 +6183,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>210</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>211</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -6270,20 +6239,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>211</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>213</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -6311,93 +6280,65 @@
       <c r="R41" s="51"/>
       <c r="S41" s="39"/>
     </row>
-    <row r="42" spans="1:19" s="75" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="73"/>
-      <c r="B42" s="47">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>182</v>
-      </c>
-      <c r="D42" s="51"/>
-      <c r="E42" s="51"/>
-      <c r="F42" s="51"/>
-      <c r="G42" s="51" t="s">
-        <v>204</v>
-      </c>
-      <c r="H42" s="51"/>
-      <c r="I42" s="51"/>
-      <c r="J42" s="51"/>
-      <c r="K42" s="51"/>
-      <c r="L42" s="51"/>
-      <c r="M42" s="51"/>
-      <c r="N42" s="51"/>
-      <c r="O42" s="61"/>
-      <c r="P42" s="52"/>
-      <c r="Q42" s="52"/>
-      <c r="R42" s="51"/>
-      <c r="S42" s="39"/>
+    <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="O42" s="85"/>
+      <c r="P42" s="85"/>
+      <c r="Q42" s="48">
+        <f>SUM(Q10:Q41)</f>
+        <v>1143.1569500000003</v>
+      </c>
+      <c r="R42" s="80"/>
+      <c r="S42" s="81"/>
     </row>
     <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="40"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="42"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="44"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="45"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="45"/>
-      <c r="L43" s="45"/>
-      <c r="M43" s="45"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
       <c r="N43" s="84" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O43" s="85"/>
       <c r="P43" s="85"/>
-      <c r="Q43" s="48">
-        <f>SUM(Q10:Q42)</f>
-        <v>1143.1569500000003</v>
-      </c>
-      <c r="R43" s="80"/>
-      <c r="S43" s="81"/>
-    </row>
-    <row r="44" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="84" t="s">
-        <v>6</v>
-      </c>
-      <c r="O44" s="85"/>
-      <c r="P44" s="85"/>
-      <c r="Q44" s="49">
-        <f>Q43/20</f>
+      <c r="Q43" s="49">
+        <f>Q42/20</f>
         <v>57.157847500000017</v>
       </c>
-      <c r="R44" s="82"/>
-      <c r="S44" s="83"/>
+      <c r="R43" s="82"/>
+      <c r="S43" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N42:P42"/>
+    <mergeCell ref="R42:S43"/>
     <mergeCell ref="N43:P43"/>
-    <mergeCell ref="R43:S44"/>
-    <mergeCell ref="N44:P44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O15" r:id="rId1"/>
@@ -6438,7 +6379,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -6681,19 +6622,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>223</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>224</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>225</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>226</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>227</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -6746,7 +6687,7 @@
         <v>51</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P10" s="38">
         <v>1.35</v>
@@ -6763,7 +6704,7 @@
     <row r="11" spans="1:19" s="75" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="73"/>
       <c r="B11" s="47">
-        <f t="shared" ref="B11:B42" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="54" t="s">
@@ -7439,19 +7380,19 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H23" s="51" t="s">
         <v>184</v>
@@ -7460,7 +7401,7 @@
         <v>172</v>
       </c>
       <c r="J23" s="51" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K23" s="51"/>
       <c r="L23" s="51">
@@ -7830,7 +7771,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -7942,7 +7883,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -8200,7 +8141,7 @@
         <v>51</v>
       </c>
       <c r="O36" s="61" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P36" s="52">
         <v>40.941549999999999</v>
@@ -8393,22 +8334,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>210</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>211</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -8449,20 +8390,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>211</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>213</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -8490,93 +8431,65 @@
       <c r="R41" s="51"/>
       <c r="S41" s="39"/>
     </row>
-    <row r="42" spans="1:19" s="75" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="73"/>
-      <c r="B42" s="47">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>182</v>
-      </c>
-      <c r="D42" s="51"/>
-      <c r="E42" s="51"/>
-      <c r="F42" s="51"/>
-      <c r="G42" s="51" t="s">
-        <v>204</v>
-      </c>
-      <c r="H42" s="51"/>
-      <c r="I42" s="51"/>
-      <c r="J42" s="51"/>
-      <c r="K42" s="51"/>
-      <c r="L42" s="51"/>
-      <c r="M42" s="51"/>
-      <c r="N42" s="51"/>
-      <c r="O42" s="61"/>
-      <c r="P42" s="52"/>
-      <c r="Q42" s="52"/>
-      <c r="R42" s="51"/>
-      <c r="S42" s="39"/>
+    <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="O42" s="85"/>
+      <c r="P42" s="85"/>
+      <c r="Q42" s="48">
+        <f>SUM(Q10:Q41)</f>
+        <v>2416.2582500000003</v>
+      </c>
+      <c r="R42" s="80"/>
+      <c r="S42" s="81"/>
     </row>
     <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="40"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="42"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="44"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="45"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="45"/>
-      <c r="L43" s="45"/>
-      <c r="M43" s="45"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
       <c r="N43" s="84" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O43" s="85"/>
       <c r="P43" s="85"/>
-      <c r="Q43" s="48">
-        <f>SUM(Q10:Q42)</f>
-        <v>2416.2582500000003</v>
-      </c>
-      <c r="R43" s="80"/>
-      <c r="S43" s="81"/>
-    </row>
-    <row r="44" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="84" t="s">
-        <v>6</v>
-      </c>
-      <c r="O44" s="85"/>
-      <c r="P44" s="85"/>
-      <c r="Q44" s="49">
-        <f>Q43/50</f>
+      <c r="Q43" s="49">
+        <f>Q42/50</f>
         <v>48.325165000000005</v>
       </c>
-      <c r="R44" s="82"/>
-      <c r="S44" s="83"/>
+      <c r="R43" s="82"/>
+      <c r="S43" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N42:P42"/>
+    <mergeCell ref="R42:S43"/>
     <mergeCell ref="N43:P43"/>
-    <mergeCell ref="R43:S44"/>
-    <mergeCell ref="N44:P44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O15" r:id="rId1"/>
@@ -8617,7 +8530,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -8860,19 +8773,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>227</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>228</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>229</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>230</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>231</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -8925,7 +8838,7 @@
         <v>101</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P10" s="38">
         <v>1.1501999999999999</v>
@@ -8942,7 +8855,7 @@
     <row r="11" spans="1:19" s="75" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="73"/>
       <c r="B11" s="47">
-        <f t="shared" ref="B11:B42" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="54" t="s">
@@ -9618,19 +9531,19 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H23" s="51" t="s">
         <v>184</v>
@@ -9639,7 +9552,7 @@
         <v>172</v>
       </c>
       <c r="J23" s="51" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -10011,7 +9924,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -10123,7 +10036,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -10381,7 +10294,7 @@
         <v>101</v>
       </c>
       <c r="O36" s="61" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P36" s="52">
         <v>36.21752</v>
@@ -10574,22 +10487,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>210</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>211</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -10630,20 +10543,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>211</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>213</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -10671,93 +10584,65 @@
       <c r="R41" s="51"/>
       <c r="S41" s="39"/>
     </row>
-    <row r="42" spans="1:19" s="75" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="73"/>
-      <c r="B42" s="47">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>182</v>
-      </c>
-      <c r="D42" s="51"/>
-      <c r="E42" s="51"/>
-      <c r="F42" s="51"/>
-      <c r="G42" s="51" t="s">
-        <v>204</v>
-      </c>
-      <c r="H42" s="51"/>
-      <c r="I42" s="51"/>
-      <c r="J42" s="51"/>
-      <c r="K42" s="51"/>
-      <c r="L42" s="51"/>
-      <c r="M42" s="51"/>
-      <c r="N42" s="51"/>
-      <c r="O42" s="61"/>
-      <c r="P42" s="52"/>
-      <c r="Q42" s="52"/>
-      <c r="R42" s="51"/>
-      <c r="S42" s="39"/>
+    <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="O42" s="85"/>
+      <c r="P42" s="85"/>
+      <c r="Q42" s="48">
+        <f>SUM(Q10:Q41)</f>
+        <v>4252.2204199999996</v>
+      </c>
+      <c r="R42" s="80"/>
+      <c r="S42" s="81"/>
     </row>
     <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="40"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="42"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="44"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="45"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="45"/>
-      <c r="L43" s="45"/>
-      <c r="M43" s="45"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
       <c r="N43" s="84" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O43" s="85"/>
       <c r="P43" s="85"/>
-      <c r="Q43" s="48">
-        <f>SUM(Q10:Q42)</f>
-        <v>4252.2204199999996</v>
-      </c>
-      <c r="R43" s="80"/>
-      <c r="S43" s="81"/>
-    </row>
-    <row r="44" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="84" t="s">
-        <v>6</v>
-      </c>
-      <c r="O44" s="85"/>
-      <c r="P44" s="85"/>
-      <c r="Q44" s="49">
-        <f>Q43/100</f>
+      <c r="Q43" s="49">
+        <f>Q42/100</f>
         <v>42.522204199999997</v>
       </c>
-      <c r="R44" s="82"/>
-      <c r="S44" s="83"/>
+      <c r="R43" s="82"/>
+      <c r="S43" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N42:P42"/>
+    <mergeCell ref="R42:S43"/>
     <mergeCell ref="N43:P43"/>
-    <mergeCell ref="R43:S44"/>
-    <mergeCell ref="N44:P44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O15" r:id="rId1"/>
@@ -10798,7 +10683,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -11041,19 +10926,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>231</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>232</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>233</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>234</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>235</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -11106,7 +10991,7 @@
         <v>501</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P10" s="38">
         <v>0.94499999999999995</v>
@@ -11123,7 +11008,7 @@
     <row r="11" spans="1:19" s="75" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="73"/>
       <c r="B11" s="47">
-        <f t="shared" ref="B11:B42" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="54" t="s">
@@ -11799,19 +11684,19 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H23" s="51" t="s">
         <v>184</v>
@@ -11820,7 +11705,7 @@
         <v>172</v>
       </c>
       <c r="J23" s="51" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -12192,7 +12077,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -12304,7 +12189,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -12562,7 +12447,7 @@
         <v>501</v>
       </c>
       <c r="O36" s="61" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P36" s="52">
         <v>34.012979999999999</v>
@@ -12755,22 +12640,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>210</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>211</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -12811,20 +12696,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>211</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>213</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -12852,93 +12737,65 @@
       <c r="R41" s="51"/>
       <c r="S41" s="39"/>
     </row>
-    <row r="42" spans="1:19" s="75" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="73"/>
-      <c r="B42" s="47">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>182</v>
-      </c>
-      <c r="D42" s="51"/>
-      <c r="E42" s="51"/>
-      <c r="F42" s="51"/>
-      <c r="G42" s="51" t="s">
-        <v>204</v>
-      </c>
-      <c r="H42" s="51"/>
-      <c r="I42" s="51"/>
-      <c r="J42" s="51"/>
-      <c r="K42" s="51"/>
-      <c r="L42" s="51"/>
-      <c r="M42" s="51"/>
-      <c r="N42" s="51"/>
-      <c r="O42" s="61"/>
-      <c r="P42" s="52"/>
-      <c r="Q42" s="52"/>
-      <c r="R42" s="51"/>
-      <c r="S42" s="39"/>
+    <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="O42" s="85"/>
+      <c r="P42" s="85"/>
+      <c r="Q42" s="48">
+        <f>SUM(Q10:Q41)</f>
+        <v>19727.451580000001</v>
+      </c>
+      <c r="R42" s="80"/>
+      <c r="S42" s="81"/>
     </row>
     <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="40"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="42"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="44"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="45"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="45"/>
-      <c r="L43" s="45"/>
-      <c r="M43" s="45"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
       <c r="N43" s="84" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O43" s="85"/>
       <c r="P43" s="85"/>
-      <c r="Q43" s="48">
-        <f>SUM(Q10:Q42)</f>
-        <v>19727.451580000001</v>
-      </c>
-      <c r="R43" s="80"/>
-      <c r="S43" s="81"/>
-    </row>
-    <row r="44" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="84" t="s">
-        <v>6</v>
-      </c>
-      <c r="O44" s="85"/>
-      <c r="P44" s="85"/>
-      <c r="Q44" s="49">
-        <f>Q43/500</f>
+      <c r="Q43" s="49">
+        <f>Q42/500</f>
         <v>39.454903160000001</v>
       </c>
-      <c r="R44" s="82"/>
-      <c r="S44" s="83"/>
+      <c r="R43" s="82"/>
+      <c r="S43" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N42:P42"/>
+    <mergeCell ref="R42:S43"/>
     <mergeCell ref="N43:P43"/>
-    <mergeCell ref="R43:S44"/>
-    <mergeCell ref="N44:P44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O15" r:id="rId1"/>
@@ -12979,7 +12836,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -13222,19 +13079,19 @@
         <v>161</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>235</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>236</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>237</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>166</v>
       </c>
       <c r="P9" s="30" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>238</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>239</v>
       </c>
       <c r="R9" s="30" t="s">
         <v>169</v>
@@ -13287,7 +13144,7 @@
         <v>1002</v>
       </c>
       <c r="O10" s="61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P10" s="38">
         <v>0.78300000000000003</v>
@@ -13304,7 +13161,7 @@
     <row r="11" spans="1:19" s="75" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="73"/>
       <c r="B11" s="47">
-        <f t="shared" ref="B11:B42" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="54" t="s">
@@ -13980,19 +13837,19 @@
         <v>14</v>
       </c>
       <c r="C23" s="54" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F23" s="51" t="s">
         <v>171</v>
       </c>
       <c r="G23" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H23" s="51" t="s">
         <v>184</v>
@@ -14001,7 +13858,7 @@
         <v>172</v>
       </c>
       <c r="J23" s="51" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K23" s="51" t="s">
         <v>172</v>
@@ -14373,7 +14230,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -14485,7 +14342,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>60</v>
@@ -14743,7 +14600,7 @@
         <v>1001</v>
       </c>
       <c r="O36" s="61" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P36" s="52">
         <v>31.493500000000001</v>
@@ -14936,22 +14793,22 @@
         <v>172</v>
       </c>
       <c r="E40" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="F40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="F40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="G40" s="51" t="s">
+      <c r="H40" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="I40" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="51" t="s">
         <v>210</v>
-      </c>
-      <c r="I40" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="J40" s="51" t="s">
-        <v>211</v>
       </c>
       <c r="K40" s="51" t="s">
         <v>172</v>
@@ -14992,20 +14849,20 @@
         <v>172</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F41" s="51"/>
       <c r="G41" s="51" t="s">
+        <v>211</v>
+      </c>
+      <c r="H41" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="H41" s="51" t="s">
-        <v>213</v>
-      </c>
       <c r="I41" s="51" t="s">
         <v>172</v>
       </c>
       <c r="J41" s="51" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K41" s="51" t="s">
         <v>172</v>
@@ -15033,93 +14890,65 @@
       <c r="R41" s="51"/>
       <c r="S41" s="39"/>
     </row>
-    <row r="42" spans="1:19" s="75" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="73"/>
-      <c r="B42" s="47">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>182</v>
-      </c>
-      <c r="D42" s="51"/>
-      <c r="E42" s="51"/>
-      <c r="F42" s="51"/>
-      <c r="G42" s="51" t="s">
-        <v>204</v>
-      </c>
-      <c r="H42" s="51"/>
-      <c r="I42" s="51"/>
-      <c r="J42" s="51"/>
-      <c r="K42" s="51"/>
-      <c r="L42" s="51"/>
-      <c r="M42" s="51"/>
-      <c r="N42" s="51"/>
-      <c r="O42" s="61"/>
-      <c r="P42" s="52"/>
-      <c r="Q42" s="52"/>
-      <c r="R42" s="51"/>
-      <c r="S42" s="39"/>
+    <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="O42" s="85"/>
+      <c r="P42" s="85"/>
+      <c r="Q42" s="48">
+        <f>SUM(Q10:Q41)</f>
+        <v>36576.230399999993</v>
+      </c>
+      <c r="R42" s="80"/>
+      <c r="S42" s="81"/>
     </row>
     <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="40"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="42"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="44"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="45"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="45"/>
-      <c r="L43" s="45"/>
-      <c r="M43" s="45"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
       <c r="N43" s="84" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O43" s="85"/>
       <c r="P43" s="85"/>
-      <c r="Q43" s="48">
-        <f>SUM(Q10:Q42)</f>
-        <v>36576.230399999993</v>
-      </c>
-      <c r="R43" s="80"/>
-      <c r="S43" s="81"/>
-    </row>
-    <row r="44" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="84" t="s">
-        <v>6</v>
-      </c>
-      <c r="O44" s="85"/>
-      <c r="P44" s="85"/>
-      <c r="Q44" s="49">
-        <f>Q43/1000</f>
+      <c r="Q43" s="49">
+        <f>Q42/1000</f>
         <v>36.576230399999993</v>
       </c>
-      <c r="R44" s="82"/>
-      <c r="S44" s="83"/>
+      <c r="R43" s="82"/>
+      <c r="S43" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N42:P42"/>
+    <mergeCell ref="R42:S43"/>
     <mergeCell ref="N43:P43"/>
-    <mergeCell ref="R43:S44"/>
-    <mergeCell ref="N44:P44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O15" r:id="rId1"/>

</xml_diff>